<commit_message>
updated tables and figures used in manuscript
</commit_message>
<xml_diff>
--- a/tables/Table1_variant_information.xlsx
+++ b/tables/Table1_variant_information.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Clade</t>
   </si>
@@ -133,10 +133,21 @@
     <t>HK.3</t>
   </si>
   <si>
-    <t>* Denotes variants with too few sequence samples available to apply the 5e-05 thresholding without breaching the 10 mutation count minimum. These variants also fail to reach 50% of the effective population. As a result, these variants have been combined into the 'transient variants'  group for all relevant analysis.</t>
-  </si>
-  <si>
-    <t>* date cutoff: June 21, 2024 because this was the last accession date for sequence data. Therefore Pirola is being cut short. Additionally, Omicron is being subset to only include sequences from its origin to the designation of a named sub-variant (kraken).</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Table 1: Variant Information. </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Population variants included in the GISAID dataset from January 2020 through June 2024. Each variant lists the associated Pango clade or Nextclade used to obtain the sequence dataset on cov-spectrum. The sequence count of each variant is included and thresholded based upon our 5x(10^-5) minimum allele frequency to obtain the minimum number of sequences with a SNP to be included in our analysis. Next, the number of SNPs at fourfold degenerate sites was calculated at this threshold. The maximum frequency within the effective population and the duration that the variant lasted. The start of the variant's duration indicates the first 3 consecutive weeks where sequences were at least 10 and the end of the variant's duration indictes the last 3 consecutive weeks where sequences were at least 10. Persistence is a value calculated by weighting the Time a variant was active by the Max Pop. Percent. The persistence value was then used to group variants into Persistent, Transient, and Other. </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -194,12 +205,71 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="18">
     <border/>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
     </border>
     <border>
       <left/>
@@ -208,55 +278,136 @@
       <bottom/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="10" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="10" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="10" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="12" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="10" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="14" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="15" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="10" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="17" fillId="2" fontId="1" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="11" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="11" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -471,7 +622,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.25"/>
+    <col customWidth="1" min="1" max="1" width="18.25"/>
     <col customWidth="1" min="2" max="2" width="9.63"/>
     <col customWidth="1" min="3" max="3" width="8.13"/>
     <col customWidth="1" min="4" max="4" width="7.13"/>
@@ -488,599 +639,597 @@
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>9</v>
+      <c r="A3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="11">
+        <v>1207325.0</v>
+      </c>
+      <c r="D3" s="12">
+        <f t="shared" ref="D3:D7" si="1">C3*0.00005</f>
+        <v>60.36625</v>
+      </c>
+      <c r="E3" s="11">
+        <v>1493.0</v>
+      </c>
+      <c r="F3" s="13">
+        <v>0.7208</v>
+      </c>
+      <c r="G3" s="14">
+        <v>44111.0</v>
+      </c>
+      <c r="H3" s="14">
+        <v>44569.0</v>
+      </c>
+      <c r="I3" s="15">
+        <f t="shared" ref="I3:I7" si="2">H3-G3</f>
+        <v>458</v>
+      </c>
+      <c r="J3" s="16">
+        <f t="shared" ref="J3:J7" si="3">F3*I3</f>
+        <v>330.1264</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="9">
-        <v>1207325.0</v>
-      </c>
-      <c r="D4" s="10">
-        <f t="shared" ref="D4:D8" si="1">C4*0.00005</f>
-        <v>60.36625</v>
-      </c>
-      <c r="E4" s="9">
-        <v>1493.0</v>
-      </c>
-      <c r="F4" s="11">
-        <v>0.7208</v>
-      </c>
-      <c r="G4" s="12">
-        <v>44111.0</v>
-      </c>
-      <c r="H4" s="12">
-        <v>44569.0</v>
-      </c>
-      <c r="I4" s="13">
-        <f t="shared" ref="I4:I8" si="2">H4-G4</f>
-        <v>458</v>
-      </c>
-      <c r="J4" s="10">
-        <f t="shared" ref="J4:J8" si="3">F4*I4</f>
-        <v>330.1264</v>
+      <c r="A4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="11">
+        <v>4526967.0</v>
+      </c>
+      <c r="D4" s="12">
+        <f t="shared" si="1"/>
+        <v>226.34835</v>
+      </c>
+      <c r="E4" s="11">
+        <v>2205.0</v>
+      </c>
+      <c r="F4" s="17">
+        <v>0.996206</v>
+      </c>
+      <c r="G4" s="14">
+        <v>44069.0</v>
+      </c>
+      <c r="H4" s="14">
+        <v>44779.0</v>
+      </c>
+      <c r="I4" s="15">
+        <f t="shared" si="2"/>
+        <v>710</v>
+      </c>
+      <c r="J4" s="16">
+        <f t="shared" si="3"/>
+        <v>707.30626</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="9">
-        <v>4526967.0</v>
-      </c>
-      <c r="D5" s="10">
+      <c r="A5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="11">
+        <v>401506.0</v>
+      </c>
+      <c r="D5" s="12">
         <f t="shared" si="1"/>
-        <v>226.34835</v>
-      </c>
-      <c r="E5" s="9">
-        <v>2205.0</v>
-      </c>
-      <c r="F5" s="14">
-        <v>0.996206</v>
-      </c>
-      <c r="G5" s="12">
-        <v>44069.0</v>
-      </c>
-      <c r="H5" s="12">
-        <v>44779.0</v>
-      </c>
-      <c r="I5" s="13">
+        <v>20.0753</v>
+      </c>
+      <c r="E5" s="11">
+        <v>2206.0</v>
+      </c>
+      <c r="F5" s="17">
+        <v>0.573118</v>
+      </c>
+      <c r="G5" s="14">
+        <v>44863.0</v>
+      </c>
+      <c r="H5" s="14">
+        <v>45369.0</v>
+      </c>
+      <c r="I5" s="15">
         <f t="shared" si="2"/>
-        <v>710</v>
-      </c>
-      <c r="J5" s="10">
+        <v>506</v>
+      </c>
+      <c r="J5" s="16">
         <f t="shared" si="3"/>
-        <v>707.30626</v>
+        <v>289.997708</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="9">
-        <v>401506.0</v>
-      </c>
-      <c r="D6" s="10">
+      <c r="A6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="11">
+        <v>6732604.0</v>
+      </c>
+      <c r="D6" s="12">
         <f t="shared" si="1"/>
-        <v>20.0753</v>
-      </c>
-      <c r="E6" s="9">
-        <v>2206.0</v>
-      </c>
-      <c r="F6" s="14">
-        <v>0.573118</v>
-      </c>
-      <c r="G6" s="12">
-        <v>44863.0</v>
-      </c>
-      <c r="H6" s="12">
-        <v>45369.0</v>
-      </c>
-      <c r="I6" s="13">
+        <v>336.6302</v>
+      </c>
+      <c r="E6" s="11">
+        <v>1325.0</v>
+      </c>
+      <c r="F6" s="13">
+        <v>0.9969</v>
+      </c>
+      <c r="G6" s="14">
+        <v>44174.0</v>
+      </c>
+      <c r="H6" s="14">
+        <v>44828.0</v>
+      </c>
+      <c r="I6" s="15">
         <f t="shared" si="2"/>
-        <v>506</v>
-      </c>
-      <c r="J6" s="10">
+        <v>654</v>
+      </c>
+      <c r="J6" s="16">
         <f t="shared" si="3"/>
-        <v>289.997708</v>
+        <v>651.9726</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="9">
-        <v>6732604.0</v>
-      </c>
-      <c r="D7" s="10">
+      <c r="A7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="11">
+        <v>261496.0</v>
+      </c>
+      <c r="D7" s="12">
         <f t="shared" si="1"/>
-        <v>336.6302</v>
-      </c>
-      <c r="E7" s="9">
-        <v>1325.0</v>
-      </c>
-      <c r="F7" s="11">
-        <v>0.9969</v>
-      </c>
-      <c r="G7" s="12">
-        <v>44174.0</v>
-      </c>
-      <c r="H7" s="12">
-        <v>44828.0</v>
-      </c>
-      <c r="I7" s="13">
+        <v>13.0748</v>
+      </c>
+      <c r="E7" s="11">
+        <v>1623.0</v>
+      </c>
+      <c r="F7" s="17">
+        <v>0.970801</v>
+      </c>
+      <c r="G7" s="14">
+        <v>45144.0</v>
+      </c>
+      <c r="H7" s="14">
+        <v>45464.0</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="2"/>
-        <v>654</v>
-      </c>
-      <c r="J7" s="10">
+        <v>320</v>
+      </c>
+      <c r="J7" s="16">
         <f t="shared" si="3"/>
-        <v>651.9726</v>
+        <v>310.65632</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="9">
-        <v>261496.0</v>
-      </c>
-      <c r="D8" s="10">
-        <f t="shared" si="1"/>
-        <v>13.0748</v>
-      </c>
-      <c r="E8" s="9">
-        <v>1623.0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0.970801</v>
-      </c>
-      <c r="G8" s="12">
-        <v>45144.0</v>
-      </c>
-      <c r="H8" s="12">
-        <v>45464.0</v>
-      </c>
-      <c r="I8" s="13">
-        <f t="shared" si="2"/>
-        <v>320</v>
-      </c>
-      <c r="J8" s="10">
-        <f t="shared" si="3"/>
-        <v>310.65632</v>
-      </c>
+      <c r="A8" s="18"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="25"/>
     </row>
     <row r="9">
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="10"/>
+      <c r="A9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="26"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="32"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="10"/>
+      <c r="A10" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="11">
+        <v>45218.0</v>
+      </c>
+      <c r="D10" s="12">
+        <f t="shared" ref="D10:D17" si="4">C10*0.00005</f>
+        <v>2.2609</v>
+      </c>
+      <c r="E10" s="11">
+        <v>1080.0</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0.025</v>
+      </c>
+      <c r="G10" s="14">
+        <v>44069.0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>44470.0</v>
+      </c>
+      <c r="I10" s="15">
+        <f t="shared" ref="I10:I17" si="5">H10-G10</f>
+        <v>401</v>
+      </c>
+      <c r="J10" s="16">
+        <f t="shared" ref="J10:J17" si="6">F10*I10</f>
+        <v>10.025</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="9">
-        <v>45218.0</v>
-      </c>
-      <c r="D11" s="10">
-        <f t="shared" ref="D11:D18" si="4">C11*0.00005</f>
-        <v>2.2609</v>
-      </c>
-      <c r="E11" s="9">
-        <v>1080.0</v>
-      </c>
-      <c r="F11" s="11">
-        <v>0.025</v>
-      </c>
-      <c r="G11" s="12">
-        <v>44069.0</v>
-      </c>
-      <c r="H11" s="12">
-        <v>44470.0</v>
-      </c>
-      <c r="I11" s="13">
-        <f t="shared" ref="I11:I18" si="5">H11-G11</f>
-        <v>401</v>
-      </c>
-      <c r="J11" s="10">
-        <f t="shared" ref="J11:J18" si="6">F11*I11</f>
-        <v>10.025</v>
+      <c r="A11" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="11">
+        <v>76367.0</v>
+      </c>
+      <c r="D11" s="12">
+        <f t="shared" si="4"/>
+        <v>3.81835</v>
+      </c>
+      <c r="E11" s="11">
+        <v>1259.0</v>
+      </c>
+      <c r="F11" s="17">
+        <v>0.095679</v>
+      </c>
+      <c r="G11" s="14">
+        <v>44111.0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>44167.0</v>
+      </c>
+      <c r="I11" s="15">
+        <f t="shared" si="5"/>
+        <v>56</v>
+      </c>
+      <c r="J11" s="16">
+        <f t="shared" si="6"/>
+        <v>5.358024</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="9">
-        <v>76367.0</v>
-      </c>
-      <c r="D12" s="10">
+      <c r="A12" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="11">
+        <v>10103.0</v>
+      </c>
+      <c r="D12" s="12">
         <f t="shared" si="4"/>
-        <v>3.81835</v>
-      </c>
-      <c r="E12" s="9">
-        <v>1259.0</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0.095679</v>
-      </c>
-      <c r="G12" s="12">
-        <v>44111.0</v>
-      </c>
-      <c r="H12" s="12">
-        <v>44167.0</v>
-      </c>
-      <c r="I12" s="13">
+        <v>0.50515</v>
+      </c>
+      <c r="E12" s="11">
+        <v>1135.0</v>
+      </c>
+      <c r="F12" s="17">
+        <v>0.0084</v>
+      </c>
+      <c r="G12" s="14">
+        <v>44195.0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>44428.0</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="5"/>
-        <v>56</v>
-      </c>
-      <c r="J12" s="10">
+        <v>233</v>
+      </c>
+      <c r="J12" s="16">
         <f t="shared" si="6"/>
-        <v>5.358024</v>
+        <v>1.9572</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="9">
-        <v>10103.0</v>
-      </c>
-      <c r="D13" s="10">
+      <c r="A13" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="11">
+        <v>134095.0</v>
+      </c>
+      <c r="D13" s="12">
         <f t="shared" si="4"/>
-        <v>0.50515</v>
-      </c>
-      <c r="E13" s="9">
-        <v>1135.0</v>
-      </c>
-      <c r="F13" s="14">
-        <v>0.0084</v>
-      </c>
-      <c r="G13" s="12">
-        <v>44195.0</v>
-      </c>
-      <c r="H13" s="12">
-        <v>44428.0</v>
-      </c>
-      <c r="I13" s="13">
+        <v>6.70475</v>
+      </c>
+      <c r="E13" s="11">
+        <v>1502.0</v>
+      </c>
+      <c r="F13" s="17">
+        <v>0.103761</v>
+      </c>
+      <c r="G13" s="14">
+        <v>44181.0</v>
+      </c>
+      <c r="H13" s="14">
+        <v>44562.0</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="5"/>
-        <v>233</v>
-      </c>
-      <c r="J13" s="10">
+        <v>381</v>
+      </c>
+      <c r="J13" s="16">
         <f t="shared" si="6"/>
-        <v>1.9572</v>
+        <v>39.532941</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="9">
-        <v>134095.0</v>
-      </c>
-      <c r="D14" s="10">
+      <c r="A14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="11">
+        <v>46078.0</v>
+      </c>
+      <c r="D14" s="12">
         <f t="shared" si="4"/>
-        <v>6.70475</v>
-      </c>
-      <c r="E14" s="9">
-        <v>1502.0</v>
-      </c>
-      <c r="F14" s="14">
-        <v>0.103761</v>
-      </c>
-      <c r="G14" s="12">
-        <v>44181.0</v>
-      </c>
-      <c r="H14" s="12">
-        <v>44562.0</v>
-      </c>
-      <c r="I14" s="13">
+        <v>2.3039</v>
+      </c>
+      <c r="E14" s="11">
+        <v>880.0</v>
+      </c>
+      <c r="F14" s="17">
+        <v>0.043532</v>
+      </c>
+      <c r="G14" s="14">
+        <v>44188.0</v>
+      </c>
+      <c r="H14" s="14">
+        <v>44428.0</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="5"/>
-        <v>381</v>
-      </c>
-      <c r="J14" s="10">
+        <v>240</v>
+      </c>
+      <c r="J14" s="16">
         <f t="shared" si="6"/>
-        <v>39.532941</v>
+        <v>10.44768</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="9">
-        <v>46078.0</v>
-      </c>
-      <c r="D15" s="10">
+      <c r="A15" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="11">
+        <v>7841.0</v>
+      </c>
+      <c r="D15" s="12">
         <f t="shared" si="4"/>
-        <v>2.3039</v>
-      </c>
-      <c r="E15" s="9">
-        <v>880.0</v>
-      </c>
-      <c r="F15" s="14">
-        <v>0.043532</v>
-      </c>
-      <c r="G15" s="12">
-        <v>44188.0</v>
-      </c>
-      <c r="H15" s="12">
-        <v>44428.0</v>
-      </c>
-      <c r="I15" s="13">
+        <v>0.39205</v>
+      </c>
+      <c r="E15" s="11">
+        <v>1078.0</v>
+      </c>
+      <c r="F15" s="17">
+        <v>0.010878</v>
+      </c>
+      <c r="G15" s="14">
+        <v>44218.0</v>
+      </c>
+      <c r="H15" s="14">
+        <v>44372.0</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="5"/>
-        <v>240</v>
-      </c>
-      <c r="J15" s="10">
+        <v>154</v>
+      </c>
+      <c r="J15" s="16">
         <f t="shared" si="6"/>
-        <v>10.44768</v>
+        <v>1.675212</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="9">
-        <v>7841.0</v>
-      </c>
-      <c r="D16" s="10">
+      <c r="A16" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="11">
+        <v>11693.0</v>
+      </c>
+      <c r="D16" s="12">
         <f t="shared" si="4"/>
-        <v>0.39205</v>
-      </c>
-      <c r="E16" s="9">
-        <v>1078.0</v>
-      </c>
-      <c r="F16" s="14">
-        <v>0.010878</v>
-      </c>
-      <c r="G16" s="12">
-        <v>44218.0</v>
-      </c>
-      <c r="H16" s="12">
-        <v>44372.0</v>
-      </c>
-      <c r="I16" s="13">
+        <v>0.58465</v>
+      </c>
+      <c r="E16" s="11">
+        <v>1420.0</v>
+      </c>
+      <c r="F16" s="17">
+        <v>0.009633</v>
+      </c>
+      <c r="G16" s="14">
+        <v>44204.0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>44512.0</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="5"/>
-        <v>154</v>
-      </c>
-      <c r="J16" s="10">
+        <v>308</v>
+      </c>
+      <c r="J16" s="16">
         <f t="shared" si="6"/>
-        <v>1.675212</v>
-      </c>
+        <v>2.966964</v>
+      </c>
+      <c r="N16" s="34"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="9">
-        <v>11693.0</v>
-      </c>
-      <c r="D17" s="10">
+      <c r="A17" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="11">
+        <v>17480.0</v>
+      </c>
+      <c r="D17" s="12">
         <f t="shared" si="4"/>
-        <v>0.58465</v>
-      </c>
-      <c r="E17" s="9">
-        <v>1420.0</v>
-      </c>
-      <c r="F17" s="14">
-        <v>0.009633</v>
-      </c>
-      <c r="G17" s="12">
-        <v>44204.0</v>
-      </c>
-      <c r="H17" s="12">
-        <v>44512.0</v>
-      </c>
-      <c r="I17" s="13">
+        <v>0.874</v>
+      </c>
+      <c r="E17" s="11">
+        <v>1621.0</v>
+      </c>
+      <c r="F17" s="17">
+        <v>0.012491</v>
+      </c>
+      <c r="G17" s="14">
+        <v>44253.0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>44540.0</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="5"/>
-        <v>308</v>
-      </c>
-      <c r="J17" s="10">
+        <v>287</v>
+      </c>
+      <c r="J17" s="16">
         <f t="shared" si="6"/>
-        <v>2.966964</v>
+        <v>3.584917</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="9">
-        <v>17480.0</v>
-      </c>
-      <c r="D18" s="10">
-        <f t="shared" si="4"/>
-        <v>0.874</v>
-      </c>
-      <c r="E18" s="9">
-        <v>1621.0</v>
-      </c>
-      <c r="F18" s="14">
-        <v>0.012491</v>
-      </c>
-      <c r="G18" s="12">
-        <v>44253.0</v>
-      </c>
-      <c r="H18" s="12">
-        <v>44540.0</v>
-      </c>
-      <c r="I18" s="13">
-        <f t="shared" si="5"/>
-        <v>287</v>
-      </c>
-      <c r="J18" s="10">
-        <f t="shared" si="6"/>
-        <v>3.584917</v>
-      </c>
+      <c r="A18" s="18"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="25"/>
     </row>
     <row r="19">
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="10"/>
+      <c r="A19" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="32"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="10"/>
+      <c r="A20" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="20">
+        <v>40179.0</v>
+      </c>
+      <c r="D20" s="20">
+        <f>C20*0.00005</f>
+        <v>2.00895</v>
+      </c>
+      <c r="E20" s="20">
+        <v>1994.0</v>
+      </c>
+      <c r="F20" s="22">
+        <v>0.129022</v>
+      </c>
+      <c r="G20" s="23">
+        <v>45095.0</v>
+      </c>
+      <c r="H20" s="23">
+        <v>45397.0</v>
+      </c>
+      <c r="I20" s="24">
+        <f>H20-G20</f>
+        <v>302</v>
+      </c>
+      <c r="J20" s="25">
+        <f>F20*I20</f>
+        <v>38.964644</v>
+      </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="9">
-        <v>40179.0</v>
-      </c>
-      <c r="D21" s="9">
-        <f>C21*0.00005</f>
-        <v>2.00895</v>
-      </c>
-      <c r="E21" s="9">
-        <v>1994.0</v>
-      </c>
-      <c r="F21" s="14">
-        <v>0.129022</v>
-      </c>
-      <c r="G21" s="12">
-        <v>45095.0</v>
-      </c>
-      <c r="H21" s="12">
-        <v>45397.0</v>
-      </c>
-      <c r="I21" s="13">
-        <f>H21-G21</f>
-        <v>302</v>
-      </c>
-      <c r="J21" s="10">
-        <f>F21*I21</f>
-        <v>38.964644</v>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="36" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24" ht="62.25" customHeight="1">
-      <c r="A24" s="17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" ht="47.25" customHeight="1">
-      <c r="A25" s="18" t="s">
-        <v>41</v>
-      </c>
-    </row>
+    <row r="23" ht="15.0" customHeight="1"/>
+    <row r="24" ht="16.5" customHeight="1"/>
+    <row r="25"/>
     <row r="26"/>
     <row r="27"/>
     <row r="28"/>
@@ -2055,11 +2204,9 @@
     <row r="997"/>
     <row r="998"/>
     <row r="999"/>
-    <row r="1000"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A25:J25"/>
+  <mergeCells count="1">
+    <mergeCell ref="A22:J29"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>